<commit_message>
feat: scan avancado genai
</commit_message>
<xml_diff>
--- a/OCR_Chaves/chaves_extraidas_final.xlsx
+++ b/OCR_Chaves/chaves_extraidas_final.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,48 +443,156 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IMG_0121.jpg</t>
+          <t>WhatsApp Image 2025-06-06 at 12.23.27.jpeg</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7NWXP-BBFGB-36W3R-GY387-T3BP6</t>
+          <t>MMN9V-TGXP4-B7YKX-2K6YP-HH66T</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IMG_0121.jpg</t>
+          <t>WhatsApp Image 2025-06-06 at 12.23.27.jpeg</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GYRFQ-GTNQJ-G7X4K-QQBCR-VMH26</t>
+          <t>33G9N-TJYJW-FVTPX-KMKF4-TVJXG</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IMG_0121.jpg</t>
+          <t>WhatsApp Image 2025-06-06 at 12.23.27.jpeg</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NCKM6-93VT7-D64WF-2X9VK-MG9TT</t>
+          <t>PF4JN-7VG89-KBBJH-V7CRX-CDKTT</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IMG_0121.jpg</t>
+          <t>WhatsApp Image 2025-06-06 at 12.23.27.jpeg</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>9NR6R-WV8RM-2BF8P-83KDM-3GPKG</t>
+          <t>G6DQH-3PN34-XGJJJ-79MC7-9BT6T</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2025-06-06 at 12.23.27.jpeg</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>R7B4Y-GNRXC-2DVP4-KYD7J-QDBP6</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2025-06-06 at 12.23.27.jpeg</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>JCXG2-NTVYK-HMM3Y-9R7MG-HFR9G</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2025-06-06 at 12.23.27.jpeg</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BR9CX-68N4X-JDK99-C2TWX-MG9TT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2025-06-06 at 12.23.29.jpeg</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BOXHN-4H3GP-26WQW-42KTP-MP2KG</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2025-06-06 at 12.23.29.jpeg</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>J6KNY-WFMTR-V87V2-BKVKK-T83GT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2025-06-06 at 12.23.29.jpeg</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HANQ6-WPGJ8-W4KYT-MFKM4-DJ3GT</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2025-06-06 at 12.23.29.jpeg</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TDDPG-7NX89-DY987-9XKYD-TCQGT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2025-06-06 at 12.23.29.jpeg</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SHN3M-Q4CWK-YX6XJ-VKBW7-8HV26</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2025-06-06 at 12.23.29.jpeg</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>KPBPR-NWY9R-QY4GP-X2979-JXCKG</t>
         </is>
       </c>
     </row>

</xml_diff>